<commit_message>
fix(druga-mila): align formatka columns with Sierpień uwagi layout
</commit_message>
<xml_diff>
--- a/data/druga-mila.xlsx
+++ b/data/druga-mila.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:D56"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -418,9 +418,6 @@
       <c r="D1" s="1" t="str">
         <v xml:space="preserve">Typ </v>
       </c>
-      <c r="E1" s="1" t="str">
-        <v>Wg harmonogramu</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
@@ -435,9 +432,6 @@
       <c r="D2" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E2" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
@@ -452,9 +446,6 @@
       <c r="D3" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E3" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
@@ -469,9 +460,6 @@
       <c r="D4" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E4" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
@@ -486,9 +474,6 @@
       <c r="D5" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E5" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
@@ -503,9 +488,6 @@
       <c r="D6" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E6" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="str">
@@ -520,9 +502,6 @@
       <c r="D7" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E7" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="str">
@@ -537,9 +516,6 @@
       <c r="D8" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E8" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="str">
@@ -554,9 +530,6 @@
       <c r="D9" s="1" t="str">
         <v>BOLĘCIN</v>
       </c>
-      <c r="E9" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="str">
@@ -571,9 +544,6 @@
       <c r="D10" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E10" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="str">
@@ -588,9 +558,6 @@
       <c r="D11" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E11" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="str">
@@ -605,9 +572,6 @@
       <c r="D12" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E12" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="str">
@@ -622,9 +586,6 @@
       <c r="D13" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E13" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="str">
@@ -639,9 +600,6 @@
       <c r="D14" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E14" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="str">
@@ -656,9 +614,6 @@
       <c r="D15" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E15" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="str">
@@ -673,9 +628,6 @@
       <c r="D16" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E16" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="str">
@@ -690,9 +642,6 @@
       <c r="D17" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E17" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="str">
@@ -707,9 +656,6 @@
       <c r="D18" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E18" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="str">
@@ -724,9 +670,6 @@
       <c r="D19" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E19" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="str">
@@ -741,9 +684,6 @@
       <c r="D20" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E20" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="str">
@@ -758,9 +698,6 @@
       <c r="D21" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E21" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="str">
@@ -775,9 +712,6 @@
       <c r="D22" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E22" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="str">
@@ -792,9 +726,6 @@
       <c r="D23" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E23" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="str">
@@ -809,9 +740,6 @@
       <c r="D24" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E24" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="str">
@@ -826,9 +754,6 @@
       <c r="D25" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E25" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="str">
@@ -843,9 +768,6 @@
       <c r="D26" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E26" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="str">
@@ -860,9 +782,6 @@
       <c r="D27" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E27" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="str">
@@ -877,9 +796,6 @@
       <c r="D28" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E28" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="str">
@@ -894,9 +810,6 @@
       <c r="D29" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E29" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="str">
@@ -911,9 +824,6 @@
       <c r="D30" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E30" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="str">
@@ -928,9 +838,6 @@
       <c r="D31" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E31" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="str">
@@ -945,9 +852,6 @@
       <c r="D32" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E32" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="str">
@@ -962,9 +866,6 @@
       <c r="D33" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E33" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="str">
@@ -979,9 +880,6 @@
       <c r="D34" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E34" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="str">
@@ -996,9 +894,6 @@
       <c r="D35" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E35" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="str">
@@ -1013,9 +908,6 @@
       <c r="D36" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E36" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="str">
@@ -1030,9 +922,6 @@
       <c r="D37" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E37" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="str">
@@ -1047,9 +936,6 @@
       <c r="D38" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E38" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="str">
@@ -1064,9 +950,6 @@
       <c r="D39" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E39" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="str">
@@ -1081,9 +964,6 @@
       <c r="D40" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E40" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="str">
@@ -1098,9 +978,6 @@
       <c r="D41" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E41" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="str">
@@ -1115,9 +992,6 @@
       <c r="D42" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E42" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="str">
@@ -1132,9 +1006,6 @@
       <c r="D43" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E43" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="str">
@@ -1149,9 +1020,6 @@
       <c r="D44" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E44" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="str">
@@ -1166,9 +1034,6 @@
       <c r="D45" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E45" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="str">
@@ -1183,9 +1048,6 @@
       <c r="D46" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E46" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="str">
@@ -1200,9 +1062,6 @@
       <c r="D47" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E47" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="str">
@@ -1217,9 +1076,6 @@
       <c r="D48" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E48" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="str">
@@ -1234,9 +1090,6 @@
       <c r="D49" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E49" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="str">
@@ -1251,9 +1104,6 @@
       <c r="D50" s="1" t="str">
         <v>PLAC</v>
       </c>
-      <c r="E50" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="str">
@@ -1268,9 +1118,6 @@
       <c r="D51" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E51" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="str">
@@ -1285,9 +1132,6 @@
       <c r="D52" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E52" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="str">
@@ -1302,9 +1146,6 @@
       <c r="D53" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E53" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="str">
@@ -1319,9 +1160,6 @@
       <c r="D54" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E54" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="str">
@@ -1336,9 +1174,6 @@
       <c r="D55" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E55" s="1" t="str">
-        <v/>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="str">
@@ -1353,13 +1188,10 @@
       <c r="D56" s="1" t="str">
         <v>CD</v>
       </c>
-      <c r="E56" s="1" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D56"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>